<commit_message>
feat(public): small table update.
</commit_message>
<xml_diff>
--- a/benchmarks/slm_flow_experiments.xlsx
+++ b/benchmarks/slm_flow_experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Михаил\Desktop\itmo_slm_flow\benchmarks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0DBC40-E1BD-46E9-B4DB-32AB3454B4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D2F11B-8F3B-4C0B-8DB3-1C1E825A95B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{010289B6-1AE1-47BB-8601-D8A41DEE1EE9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="182">
   <si>
     <t>модель</t>
   </si>
@@ -512,30 +512,9 @@
     <t>Аналог - RouteLLM</t>
   </si>
   <si>
-    <t>mf (matrix factorization)</t>
-  </si>
-  <si>
-    <t>0.68</t>
-  </si>
-  <si>
-    <t>0.57</t>
-  </si>
-  <si>
-    <t>0.25</t>
-  </si>
-  <si>
-    <t>0.30</t>
-  </si>
-  <si>
     <t>0.38</t>
   </si>
   <si>
-    <t>0.62</t>
-  </si>
-  <si>
-    <t>0.71</t>
-  </si>
-  <si>
     <t>sw_ranking</t>
   </si>
   <si>
@@ -572,9 +551,6 @@
     <t>0.31</t>
   </si>
   <si>
-    <t>2.423</t>
-  </si>
-  <si>
     <t>2.411</t>
   </si>
   <si>
@@ -596,9 +572,6 @@
     <t>0.146</t>
   </si>
   <si>
-    <t>3.441</t>
-  </si>
-  <si>
     <t>3.408</t>
   </si>
   <si>
@@ -609,9 +582,6 @@
   </si>
   <si>
     <t>2.231</t>
-  </si>
-  <si>
-    <t>4.531</t>
   </si>
   <si>
     <t>4.493</t>
@@ -778,6 +748,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -787,20 +762,15 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="21" fontId="2" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1137,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81177C81-A37B-473A-86B9-20BCFF158C64}">
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
@@ -1489,22 +1459,22 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="8"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="11"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1675,200 +1645,158 @@
       <c r="N13" s="1"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="14"/>
+      <c r="N14" s="14"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="D15" s="11" t="s">
+      <c r="C15" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="I15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="K15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="15" t="s">
-        <v>182</v>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="8" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="C16" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="K16" s="11" t="s">
+      <c r="K16" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="15" t="s">
-        <v>182</v>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="8" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="J17" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C17" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="K17" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="L17" s="11" t="s">
+      <c r="K17" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="L17" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="M17" s="11" t="s">
+      <c r="M17" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="N17" s="15"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="M18" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="N18" s="15" t="s">
-        <v>183</v>
+      <c r="N17" s="8" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -1993,110 +1921,84 @@
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="D31" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
+      <c r="A32" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F32" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="D32" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="F32" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="E33" s="15" t="s">
+      <c r="B33" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="F33" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="G33" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="G34" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="H34" s="15" t="s">
+      <c r="H33" s="8" t="s">
         <v>154</v>
       </c>
     </row>

</xml_diff>